<commit_message>
added check binomial to alternate names
</commit_message>
<xml_diff>
--- a/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-30.xlsx
+++ b/splists_out/needs_revision/BCI_SPECIES_POSSIBLY_WOODY_2026-03-30.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X62"/>
+  <dimension ref="A1:X61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -5368,7 +5368,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5378,17 +5378,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2539336</t>
+          <t>168181</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1012528-1</t>
+          <t>963361-1</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5398,52 +5398,57 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum var. pinnatum</t>
+          <t>Palicourea tonduzii</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum</t>
+          <t>Palicourea tonduzii</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Fabaceae</t>
+          <t>Rubiaceae</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>(K.Krause) A.C.Berger</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>3240068</t>
+          <t>526435</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>77213974-1</t>
+          <t>77162934-1</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>77213974-1</t>
+          <t>77162934-1</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>tree</t>
+          <t>subshrub or shrub</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum subsp. polystachyum</t>
+          <t>Psychotria guapilensis</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Platymiscium pinnatum (Jacq.) Dugand sensu Croat (1978)</t>
+          <t>Cephaelis discolor Pol.</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
       <c r="T56" t="b">
@@ -5456,7 +5461,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5466,32 +5471,32 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>168181</t>
+          <t>179388</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>963361-1</t>
+          <t>764727-1</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Synonym</t>
+          <t>Accepted</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Palicourea tonduzii</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Palicourea tonduzii</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -5501,22 +5506,22 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>(K.Krause) A.C.Berger</t>
+          <t>(L.f.) A.Rich.</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>526435</t>
+          <t>179388</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>77162934-1</t>
+          <t>764727-1</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>77162934-1</t>
+          <t>764727-1</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -5526,12 +5531,12 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Psychotria guapilensis</t>
+          <t>Ronabea emetica</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Cephaelis discolor Pol.</t>
+          <t>Psychotria emetica L.f. (Croat 1978; Correa et al. 2004)</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -5549,7 +5554,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5559,17 +5564,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>179388</t>
+          <t>3125397</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>764727-1</t>
+          <t>987251-1</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5579,37 +5584,37 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Rubiaceae</t>
+          <t>Asteraceae</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>(L.f.) A.Rich.</t>
+          <t>(Fenzl) Kuntze</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>179388</t>
+          <t>3125397</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>764727-1</t>
+          <t>987251-1</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>764727-1</t>
+          <t>987251-1</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5619,17 +5624,17 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Ronabea emetica</t>
+          <t>Schistocarpha eupatorioides</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Psychotria emetica L.f. (Croat 1978; Correa et al. 2004)</t>
+          <t>Schistocarpha oppositifolia (Kuntze) Rydb.</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
       <c r="T58" t="b">
@@ -5642,27 +5647,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Garwood2009</t>
+          <t>Zotz</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>3125397</t>
+          <t>199060</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>987251-1</t>
+          <t>89152-1</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5672,61 +5677,61 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
+          <t>Syngonium podophyllum</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Asteraceae</t>
+          <t>Araceae</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>(Fenzl) Kuntze</t>
+          <t>Schott</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>3125397</t>
+          <t>199060</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>987251-1</t>
+          <t>89152-1</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>987251-1</t>
+          <t>89152-1</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>subshrub or shrub</t>
+          <t>liana</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Schistocarpha eupatorioides</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>Schistocarpha oppositifolia (Kuntze) Rydb.</t>
+          <t>Syngonium podophyllum var. podophyllum</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Hw</t>
+          <t>E</t>
         </is>
       </c>
       <c r="T59" t="b">
         <v>0</v>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Syngonium podophyllum</t>
+        </is>
       </c>
       <c r="X59" t="b">
         <v>0</v>
@@ -5735,27 +5740,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Zotz</t>
+          <t>Garwood2009</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>199060</t>
+          <t>215102</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>89152-1</t>
+          <t>89333-1</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5765,12 +5770,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -5780,46 +5785,41 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Schott</t>
+          <t>(Jacq.) Schott</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>199060</t>
+          <t>215102</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>89152-1</t>
+          <t>89333-1</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>89152-1</t>
+          <t>89333-1</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>liana</t>
+          <t>tuberous subshrub</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Syngonium podophyllum var. podophyllum</t>
+          <t>Xanthosoma helleborifolium</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>H</t>
         </is>
       </c>
       <c r="T60" t="b">
         <v>0</v>
-      </c>
-      <c r="U60" t="inlineStr">
-        <is>
-          <t>Syngonium podophyllum</t>
-        </is>
       </c>
       <c r="X60" t="b">
         <v>0</v>
@@ -5828,7 +5828,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5838,17 +5838,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>215102</t>
+          <t>215118</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>89333-1</t>
+          <t>89347-1</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5858,12 +5858,12 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Xanthosoma mexicanum</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -5873,22 +5873,22 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>(Jacq.) Schott</t>
+          <t>Liebm.</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>215102</t>
+          <t>215118</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>89333-1</t>
+          <t>89347-1</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>89333-1</t>
+          <t>89347-1</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -5898,111 +5898,23 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Xanthosoma helleborifolium</t>
+          <t>Xanthosoma mexicanum</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Xanthosoma pilosum K.Koch &amp; Augustin (Croat 1978, Correa et al. 2004)</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Hw</t>
         </is>
       </c>
       <c r="T61" t="b">
         <v>0</v>
       </c>
       <c r="X61" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Garwood2009</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>215118</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>89347-1</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Accepted</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Araceae</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>Liebm.</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>215118</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>89347-1</t>
-        </is>
-      </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>89347-1</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>tuberous subshrub</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>Xanthosoma mexicanum</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>Xanthosoma pilosum K.Koch &amp; Augustin (Croat 1978, Correa et al. 2004)</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>Hw</t>
-        </is>
-      </c>
-      <c r="T62" t="b">
-        <v>0</v>
-      </c>
-      <c r="X62" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6454,7 +6366,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>splists_out/alternates_and_synonyms/AltNames_2026-03-29.xlsx</t>
+          <t>splists_out/alternates_and_synonyms/AltNames_2026-03-30.xlsx</t>
         </is>
       </c>
     </row>
@@ -6466,7 +6378,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>splists_out/alternates_and_synonyms/alternate_names_garwood_2026-03-29.xlsx</t>
+          <t>splists_out/alternates_and_synonyms/alternate_names_garwood_2026-03-30.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>